<commit_message>
Update STEP data model to Entity terminology
Replaced Product with Entity throughout hierarchy structure,
object types, and load order to match actual STEP setup.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -462,24 +462,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GPOHierarchy</t>
+          <t>GPO_Hierarchy_Root</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GPO Hierarchy</t>
+          <t>GPO Hierarchy Root</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Classification</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>Entity Classification</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Entity hierarchy root</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Root node for all GPO data</t>
+          <t>Root entity node for all GPO data</t>
         </is>
       </c>
     </row>
@@ -499,18 +503,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Entity Classification</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GPOHierarchy</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>GPO_Hierarchy_Root</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GPO Types</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>HealthTrust GPO grouping node</t>
+          <t>HealthTrust GPO grouping entity</t>
         </is>
       </c>
     </row>
@@ -530,18 +538,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Entity Classification</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GPOHierarchy</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>GPO_Hierarchy_Root</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GPO Types</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Premier GPO grouping node</t>
+          <t>Premier GPO grouping entity</t>
         </is>
       </c>
     </row>
@@ -561,18 +573,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Entity Classification</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GPOHierarchy</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>GPO_Hierarchy_Root</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GPO Types</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Vizient GPO grouping node</t>
+          <t>Vizient GPO grouping entity</t>
         </is>
       </c>
     </row>
@@ -592,7 +608,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -602,12 +618,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>HealthTrust top parent — 399 nodes</t>
+          <t>HealthTrust top parent entities — 399 nodes</t>
         </is>
       </c>
     </row>
@@ -627,7 +643,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -637,12 +653,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Premier top parent nodes</t>
+          <t>Premier top parent entities</t>
         </is>
       </c>
     </row>
@@ -662,7 +678,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -672,12 +688,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Vizient top parent (System) nodes</t>
+          <t>Vizient top parent (System) entities</t>
         </is>
       </c>
     </row>
@@ -697,7 +713,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -707,12 +723,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>HealthTrust direct parent — 6159 nodes</t>
+          <t>HealthTrust direct parent entities — 6159 nodes</t>
         </is>
       </c>
     </row>
@@ -732,7 +748,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -742,12 +758,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Premier direct parent nodes</t>
+          <t>Premier direct parent entities</t>
         </is>
       </c>
     </row>
@@ -767,7 +783,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -777,12 +793,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>GPO_Member</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Vizient direct parent nodes</t>
+          <t>Vizient direct parent entities</t>
         </is>
       </c>
     </row>
@@ -802,7 +818,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -817,7 +833,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>HealthTrust leaf members — 95550 nodes</t>
+          <t>HealthTrust member entities — 95550 nodes</t>
         </is>
       </c>
     </row>
@@ -837,7 +853,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -852,7 +868,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Premier leaf members</t>
+          <t>Premier member entities</t>
         </is>
       </c>
     </row>
@@ -872,7 +888,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Entity</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -887,7 +903,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Vizient leaf members</t>
+          <t>Vizient member entities</t>
         </is>
       </c>
     </row>
@@ -902,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -918,30 +934,75 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Parent Object Type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Used By</t>
+          <t>Used For</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>GPO Types</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GPO Types</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GPO_HealthTrust, GPO_Premier, GPO_Vizient classification nodes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GPO_Top_Parent</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GPO Top Parent</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Top parent entities across all 3 GPOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GPO_Direct_Parent</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GPO Direct Parent</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Direct parent entities across all 3 GPOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>GPO_Member</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>GPO Member</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>All GPOs — Top Parent, Direct Parent, Leaf Member</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Leaf member entities across all 3 GPOs</t>
         </is>
       </c>
     </row>
@@ -982,7 +1043,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Level</t>
+          <t>Entity Level</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1668,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Node Type</t>
+          <t>Entity Type</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -1632,7 +1693,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Entity Classification</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -1640,7 +1701,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GPOHierarchy must exist</t>
+          <t>GPO Hierarchy Root must exist</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1716,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -1678,7 +1739,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -1701,7 +1762,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Member</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -1724,7 +1785,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1749,7 +1810,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1774,7 +1835,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Member</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1799,7 +1860,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Top_Parent</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1824,7 +1885,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Direct_Parent</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1849,7 +1910,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>GPO_Member</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">

</xml_diff>

<commit_message>
Add Unique Key Design sheet to STEP data model
Documents ID format per GPO, deduplication strategy, reimport
behaviour, and cross-GPO isolation via prefix.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Object Types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Attributes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Load Order" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1927,4 +1928,240 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>GPO</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Native ID Field</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>STEP Entity ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Example</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Dedup Before Load</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>On Reimport</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Cross-GPO Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GPOID</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HT_&lt;GPOID&gt;</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>HT_H109794</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Yes — drop_duplicates on GPOID (removes DEA duplicates)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>STEP matches by ID and updates existing entity — no duplicate created</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>None — HT_ prefix isolates from Premier and Vizient IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Address ID</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PR_&lt;AddressID&gt;</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PR_98765</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Not needed — Address ID is already unique per row</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>STEP matches by ID and updates existing entity — no duplicate created</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>None — PR_ prefix isolates from HealthTrust and Vizient IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LIC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VZ_&lt;LIC&gt;</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VZ_A1234</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not needed — LIC is already unique per row</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>STEP matches by ID and updates existing entity — no duplicate created</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>None — VZ_ prefix isolates from HealthTrust and Premier IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>All — Top Parents</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Top Parent GPOID / Top Parent GPO ID / System ID</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HT_/PR_/VZ_ + top parent ID</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HT_H100691</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Yes — extracted with drop_duplicates on top parent ID</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>STEP matches by ID and updates existing entity — no duplicate created</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>None — prefix ensures uniqueness across GPOs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>All — Direct Parents</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Direct Parent GPOID / Direct Parent GPO ID / Parent ID</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HT_/PR_/VZ_ + direct parent ID</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HT_H200100</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Yes — extracted with drop_duplicates on direct parent ID from 3-level leaf rows</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>STEP matches by ID and updates existing entity — no duplicate created</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>None — prefix ensures uniqueness across GPOs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add GPO_Vizient_Key attribute for LIC unique key
Vizient LIC stored as GPO_Vizient_Key attribute in STEPXML.
Added GPO_ATTRIBUTE_MAP for GPO-specific attribute overrides
so LIC maps to GPO_Vizient_Key only for Vizient, not all GPOs.
Excel updated with new attribute and key attribute ID column.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1637,6 +1637,33 @@
         </is>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GPO_Vizient_Key</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>LIC (Vizient Unique Key)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>All</t>
         </is>
@@ -1936,7 +1963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1975,6 +2002,11 @@
           <t>Cross-GPO Risk</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>STEP Key Attribute ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2012,6 +2044,11 @@
           <t>None — HT_ prefix isolates from Premier and Vizient IDs</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>GPO_NativeMemberID</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2049,6 +2086,11 @@
           <t>None — PR_ prefix isolates from HealthTrust and Vizient IDs</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>GPO_NativeMemberID</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2086,6 +2128,11 @@
           <t>None — VZ_ prefix isolates from HealthTrust and Premier IDs</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>GPO_Vizient_Key</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2123,6 +2170,7 @@
           <t>None — prefix ensures uniqueness across GPOs</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2160,6 +2208,7 @@
           <t>None — prefix ensures uniqueness across GPOs</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Standardise GPO key attribute IDs
GPO_HealthTrust_Key → GPOID
GPO_Premier_Key     → Address ID (needs creating in STEP)
GPO_Vizient_Key     → LIC

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1047,16 +1047,21 @@
           <t>Entity Level</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GPO_NativeMemberID</t>
+          <t>GPO_Name2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Native Member ID</t>
+          <t>Name 2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1066,24 +1071,25 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>HealthTrust, Premier</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>All</t>
-        </is>
-      </c>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GPO_Name2</t>
+          <t>GPO_AddressType</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Name 2</t>
+          <t>Address Type</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1093,7 +1099,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>HealthTrust, Premier</t>
+          <t>Premier</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1101,16 +1107,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GPO_AddressType</t>
+          <t>GPO_Address1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Address Type</t>
+          <t>Address 1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1120,7 +1127,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Premier</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1128,16 +1135,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GPO_Address1</t>
+          <t>GPO_Address2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Address 1</t>
+          <t>Address 2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1155,16 +1163,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GPO_Address2</t>
+          <t>GPO_Address3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Address 2</t>
+          <t>Address 3</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1174,7 +1183,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>HealthTrust, Premier</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1182,16 +1191,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GPO_Address3</t>
+          <t>GPO_City</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Address 3</t>
+          <t>City</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1201,7 +1211,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HealthTrust, Premier</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1209,16 +1219,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GPO_City</t>
+          <t>GPO_State</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>State / Province</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1236,16 +1247,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GPO_State</t>
+          <t>GPO_PostalCode</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>State / Province</t>
+          <t>Postal Code</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1263,16 +1275,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GPO_PostalCode</t>
+          <t>GPO_Country</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Postal Code</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1282,7 +1295,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>HealthTrust, Premier</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1290,16 +1303,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GPO_Country</t>
+          <t>GPO_MemberStatus</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Member Status</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1317,26 +1331,27 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GPO_MemberStatus</t>
+          <t>GPO_MembershipEligibleDate</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Member Status</t>
+          <t>Membership Eligible Date</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>HealthTrust, Premier</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1344,26 +1359,27 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GPO_MembershipEligibleDate</t>
+          <t>GPO_Comments</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Membership Eligible Date</t>
+          <t>Comments</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>HealthTrust</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1371,16 +1387,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GPO_Comments</t>
+          <t>GPO_OverrideName</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Override Name</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1390,7 +1407,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>HealthTrust</t>
+          <t>Premier</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1398,16 +1415,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GPO_OverrideName</t>
+          <t>GPO_RelationshipToTopParent</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Override Name</t>
+          <t>Relationship to Top Parent</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1425,16 +1443,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GPO_RelationshipToTopParent</t>
+          <t>GPO_RelationshipToDirectParent</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Relationship to Top Parent</t>
+          <t>Relationship to Direct Parent</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1452,16 +1471,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GPO_RelationshipToDirectParent</t>
+          <t>GPO_CommittedProgramEligibility</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Relationship to Direct Parent</t>
+          <t>Committed Program Eligibility</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1479,16 +1499,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GPO_CommittedProgramEligibility</t>
+          <t>GPO_PremierGPOID</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Committed Program Eligibility</t>
+          <t>Premier GPO ID</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1506,16 +1527,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GPO_PremierGPOID</t>
+          <t>GPO_VizientMemberID</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Premier GPO ID</t>
+          <t>Vizient Member ID</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1525,7 +1547,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Premier</t>
+          <t>Vizient</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1533,16 +1555,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GPO_VizientMemberID</t>
+          <t>GPO_SupplyProgram</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Vizient Member ID</t>
+          <t>Supply Program</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1560,16 +1583,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GPO_SupplyProgram</t>
+          <t>GPO_AMCTierPricing</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Supply Program</t>
+          <t>AMC Tier Pricing</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1587,16 +1611,17 @@
           <t>Member</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GPO_AMCTierPricing</t>
+          <t>GPO_Source</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AMC Tier Pricing</t>
+          <t>GPO Source</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1606,24 +1631,25 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Vizient</t>
+          <t>All</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Member</t>
-        </is>
-      </c>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GPO_Source</t>
+          <t>GPO_HealthTrust_Key</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GPO Source</t>
+          <t>GPO HealthTrust Key</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1633,39 +1659,81 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>All</t>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Stores GPOID — gpo.GPO_Member_ID — exists in STEP</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>GPO_Premier_Key</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>GPO Premier Key</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Stores Address ID — gpo.GPO_Address_ID — NEW, needs creating in STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>GPO_Vizient_Key</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>LIC (Vizient Unique Key)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>GPO Vizient Key</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>All</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Stores LIC — gpo.LIC — exists in STEP</t>
         </is>
       </c>
     </row>
@@ -1963,7 +2031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2007,6 +2075,11 @@
           <t>STEP Key Attribute ID</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2046,7 +2119,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>GPO_NativeMemberID</t>
+          <t>GPO_HealthTrust_Key</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2166,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>GPO_NativeMemberID</t>
+          <t>GPO_Premier_Key</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>GPO_Premier_Key needs to be created in STEP</t>
         </is>
       </c>
     </row>
@@ -2133,6 +2216,11 @@
           <t>GPO_Vizient_Key</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2170,7 +2258,16 @@
           <t>None — prefix ensures uniqueness across GPOs</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2208,7 +2305,16 @@
           <t>None — prefix ensures uniqueness across GPOs</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update ATTRIBUTE_MAP to use confirmed STEP attribute IDs
Maps all GPO fields to correct loc.*, gpo.* attribute IDs.
12 existing attributes reused, 17 flagged as needing creation.
GPO key attributes updated to gpo.GPO_Member_ID, gpo.LIC, gpo.GPO_Premier_Key.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Attributes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Load Order" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2319,4 +2320,1010 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>GPO Field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Internal Field</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>STEP Attribute ID</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>STEP Attribute Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>GPO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GPOID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>native_member_id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Member_ID</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>GPO Member ID</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Address ID</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>native_member_id</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Premier_Key</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GPO Premier Key</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LIC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>native_member_id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>gpo.LIC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LIC</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Name1 / Name 1 / Member Name</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>name1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>(STEP Entity Name)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Name2 / Name 2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>name2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>gpo.Name_2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Name 2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HT, Premier</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Override Name</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>override_name</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>gpo.Override_Name</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Override Name</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>address_type</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>gpo.Address_Type</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Address1 / Address 1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>address1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>loc.Address_Line_1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Address Line 1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Address2 / Address 2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>address2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>loc.Address_Line_2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Address Line 2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Address3 / Address 3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>address3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>loc.Address_Line_3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Address Line 3</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HT, Premier</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>loc.Address_City</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Address City</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>State/Province / State</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>loc.Address_State</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Address State</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Postal Code / Zip Code</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>postal_code</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>loc.Address_Postal_Code</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Address Postal Code</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>loc.Address_Country</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Address Country</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>HT, Premier</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Member Status</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>member_status</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>gpo.Member_Status</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Member Status</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>HT, Premier</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Membership Eligible/Start Date</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>membership_eligible_date</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>gpo.Membership_Eligible_Date</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Membership Eligible Date</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>comments</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>gpo.Comments</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GPO ID</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>premier_gpo_id</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>gpo.Premier_GPO_ID</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Premier GPO ID</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Relationship to Top Parent</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>relationship_to_top_parent</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>gpo.Relationship_To_Top_Parent</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Relationship to Top Parent</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Relationship to Direct Parent</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>relationship_to_direct_parent</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>gpo.Relationship_To_Direct_Parent</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Relationship to Direct Parent</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Committed Program Eligibility</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>committed_program_eligibility</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>gpo.Committed_Program_Eligibility</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Committed Program Eligibility</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>affiliation_1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>gpo.Aggregation_Affiliation_1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 1</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>affiliation_2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>gpo.Aggregation_Affiliation_2</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 2</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>affiliation_3</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>gpo.Aggregation_Affiliation_3</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Aggregation Affiliation 3</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Member ID</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>vizient_member_id</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>gpo.Vizient_Member_ID</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Vizient Member ID</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Supply Program</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>supply_program</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>gpo.Supply_Program</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Supply Program</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AMC Tier Pricing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>amc_tier_pricing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>gpo.AMC_Tier_Pricing</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>AMC Tier Pricing</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Vizient Group 1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>group_1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>gpo.Vizient_Group_1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Vizient Group 1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Vizient Group 2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>group_2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>gpo.Vizient_Group_2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Vizient Group 2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Vizient Group 3</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>group_3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>gpo.Vizient_Group_3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Vizient Group 3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mark gpo.Vizient_Group_1/2/3 as existing in STEP
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3255,7 +3255,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Needs Creating</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Needs Creating</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Needs Creating</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Map Premier GPO ID to existing gpo.GPO_Member_ID attribute
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2920,7 +2920,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>gpo.Premier_GPO_ID</t>
+          <t>gpo.GPO_Member_ID</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Needs Creating</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add GPO Reference Type sheet to data model
Documents the GPO reference type linking customer entities
(Customer_Business_Unit, Halyard_Customer, Medical_Distribution_Customer)
to GPO target types (GPO_Top_Parent, GPO_Direct_Parent, GPO_Member).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Load Order" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Reference Type" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3326,4 +3327,178 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reference Type</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GPO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GPO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Links customer entities to GPO member entities</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Valid Source Types (Customer side)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Customer_Business_Unit</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Customer Business Unit</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Halyard_Customer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Halyard Customer Account</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Medical_Distribution_Customer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Medical Distribution Customer Account</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Valid Target Types (GPO side)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GPO_Top_Parent</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GPO Top Parent</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Root level GPO entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GPO_Direct_Parent</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GPO Direct Parent</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mid-level GPO entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GPO_Member</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GPO Member</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Leaf level GPO entity</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Document auto-matching rules for GPO reference type
GPO reference auto-created by matching customer key fields
to GPO entity key attributes:
  gpo.GPO_Member_ID → HealthTrust
  gpo.LIC           → Vizient
  gpo.GPO_Premier_Key → Premier

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3335,7 +3335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,7 +3356,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Matching Logic</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Links customer entities to GPO member entities</t>
+          <t>Auto-created by matching customer key to GPO entity key attribute</t>
         </is>
       </c>
     </row>
@@ -3456,11 +3456,7 @@
           <t>GPO Top Parent</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Root level GPO entity</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
@@ -3474,11 +3470,7 @@
           <t>GPO Direct Parent</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Mid-level GPO entity</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
@@ -3492,9 +3484,69 @@
           <t>GPO Member</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Leaf level GPO entity</t>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Auto-Matching Rules</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Member_ID</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GPO Member ID</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Customer GPO Member ID → matches HealthTrust GPO entity (gpo.GPO_Member_ID)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>gpo.LIC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LIC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Customer LIC → matches Vizient GPO entity (gpo.LIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Premier_Key</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GPO Premier Key</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Customer Address ID → matches Premier GPO entity (gpo.GPO_Premier_Key)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add gpo.Member_Date attribute for Vizient Member Date field
Vizient uses Member Date separately from gpo.Membership_Eligible_Date
used by HealthTrust and Premier.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2329,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>HealthTrust, Premier</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3321,6 +3321,38 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Member Date</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>membership_eligible_date</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>gpo.Member_Date</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Member Date</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Share gpo.Member_Date between Premier and Vizient date fields
HealthTrust → gpo.Membership_Eligible_Date (exists)
Premier     → gpo.Member_Date (Membership Start Date, needs creating)
Vizient     → gpo.Member_Date (Member Date, needs creating)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2329,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2847,7 +2847,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Membership Eligible/Start Date</t>
+          <t>Membership Eligible Date</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HealthTrust, Premier</t>
+          <t>HealthTrust</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3351,6 +3351,38 @@
         </is>
       </c>
       <c r="F32" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Membership Start Date</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>membership_eligible_date</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>gpo.Member_Date</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Member Date</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>

</xml_diff>

<commit_message>
Use gpo.Membership_Eligible_Date for all 3 GPOs
Single shared attribute for HT/Premier/Vizient membership dates.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2329,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HealthTrust</t>
+          <t>All</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3321,70 +3321,6 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>Exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Member Date</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>membership_eligible_date</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>gpo.Member_Date</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Member Date</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Vizient</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Membership Start Date</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>membership_eligible_date</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>gpo.Member_Date</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Member Date</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Premier</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add affiliation start/end date attributes (1, 2, 3) for Premier
- Added 6 new STEP attribute IDs to ATTRIBUTE_MAP in gpo_to_stepxml.py:
  gpo.Affiliation_Start_Date_1/2/3 and gpo.Affiliation_End_Date_1/2/3
- Added matching rows to Attribute Mapping sheet in step_data_model.xlsx,
  marked as Needs Creating, inserted after Aggregation Affiliation 3

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -32,12 +32,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,8 +58,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -483,7 +492,6 @@
           <t>Entity hierarchy root</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Root entity node for all GPO data</t>
@@ -1081,7 +1089,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1109,7 +1116,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1137,7 +1143,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1165,7 +1170,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1193,7 +1197,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1221,7 +1224,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1249,7 +1251,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1277,7 +1278,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1305,7 +1305,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1333,7 +1332,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1361,7 +1359,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1389,7 +1386,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1417,7 +1413,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1445,7 +1440,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1473,7 +1467,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1501,7 +1494,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1529,7 +1521,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1557,7 +1548,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1585,7 +1575,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1613,7 +1602,6 @@
           <t>Member</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1641,7 +1629,6 @@
           <t>All</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2329,7 +2316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3133,192 +3120,384 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 1</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_1_start</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_Start_Date_1</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 1</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 1</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_1_end</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_End_Date_1</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 1</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 2</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_2_start</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_Start_Date_2</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 2</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 2</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_2_end</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_End_Date_2</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 2</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 3</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_3_start</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_Start_Date_3</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation Start Date 3</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 3</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>affiliation_3_end</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>gpo.Affiliation_End_Date_3</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="inlineStr">
+        <is>
+          <t>Affiliation End Date 3</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>Needs Creating</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Member ID</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>vizient_member_id</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>gpo.Vizient_Member_ID</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Vizient Member ID</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>supply_program</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>gpo.Supply_Program</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>amc_tier_pricing</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>gpo.AMC_Tier_Pricing</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Vizient Group 1</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>group_1</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_1</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Vizient Group 1</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Vizient Group 2</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>group_2</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_2</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Vizient Group 2</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Vizient Group 3</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>group_3</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_3</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Vizient Group 3</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
@@ -3382,12 +3561,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3404,10 +3578,8 @@
           <t>Customer Business Unit</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Halyard_Customer</t>
@@ -3418,10 +3590,8 @@
           <t>Halyard Customer Account</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Medical_Distribution_Customer</t>
@@ -3432,14 +3602,8 @@
           <t>Medical Distribution Customer Account</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3456,10 +3620,8 @@
           <t>GPO Top Parent</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>GPO_Direct_Parent</t>
@@ -3470,10 +3632,8 @@
           <t>GPO Direct Parent</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>GPO_Member</t>
@@ -3484,14 +3644,8 @@
           <t>GPO Member</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3515,7 +3669,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>gpo.LIC</t>
@@ -3533,7 +3686,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>gpo.GPO_Premier_Key</t>

</xml_diff>

<commit_message>
Add Potential Gaps sheet to step_data_model.xlsx
15 items covering: missing field mappings (HT/Vizient), program/group
reference types not yet defined in STEP, orphaned parent synthesis,
unique key setup, date format handling, large file chunking, DEA data,
STEP attribute data types, and re-import idempotency.
Each row tagged High / Medium / Low with a recommended action.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Reference Type" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Potential Gaps" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +32,12 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +48,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+        <bgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0E0"/>
+        <bgColor rgb="00FFE0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,10 +81,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3561,7 +3596,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3603,7 +3637,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3645,7 +3678,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3699,6 +3731,510 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>Customer Address ID → matches Premier GPO entity (gpo.GPO_Premier_Key)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Gap / Risk</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>GPO(s) Affected</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Attribute — Programs</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>AscenDrive / KIINDO / SURPASS program start &amp; end dates are written as CrossReference elements in STEPXML, but no STEP Attribute IDs are defined for them. STEP may not have these object types or reference types configured.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Confirm with STEP admin whether programs are stored as child entities or as attributes. Create object types / reference types in STEP before loading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Attribute — Groups</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Vizient Group 1/2/3 are emitted as CrossReference elements but no corresponding STEP Reference Type is defined for member groups.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Define a MemberGroup reference type in STEP or convert groups to multi-value attributes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Missing Fields — HealthTrust</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Several HealthTrust source columns are not mapped to STEP: Phone, Fax, GLN, HIN, COID, CCN, Organizational Status, Class of Trade, Facility Type, Licensed Beds, Pharmacy Eligible/Ineligible Date, HRSA Flag, HRSA Number, HRSA Eligible/Ineligible Date, DSH Flag, AdvantageTrust Flag, Membership Ineligible Date, Relationship to GPO.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Confirm which of these are required in STEP. Create attributes and add to ATTRIBUTE_MAP for any that are needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Missing Fields — Vizient</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Vizient source columns not mapped: Member Phone, Facility Type, Facility Category, Provista Member, Excelerate Member, Rx Group. No member_status equivalent confirmed for Vizient.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Confirm with business which Vizient fields are needed. Add attribute mappings accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Hierarchy — Orphaned Parents</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Top parent or direct parent IDs referenced by child rows may not exist as their own rows in the source file. The script synthesizes implied top parents (Pass 1b) but does not synthesize implied direct parents.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Add Pass 1b-equivalent logic for implied direct parents. Validate after load that all parent FK references resolve in STEP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Hierarchy — Cross-GPO Duplicates</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>STEP entity IDs are prefixed (HT_, PR_, VZ_) to prevent collision, but the same physical facility may appear in multiple GPOs under different IDs with no cross-reference linking them.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Consider a GLN or HIN-based deduplication pass across GPOs, or a manual review process to identify overlapping facilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Date Format</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Source Excel date columns may be read as Python datetime objects or as strings. STEP expects ISO 8601 format (YYYY-MM-DD). Inconsistent source formats could cause silent load failures.</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Validate format_date() handles all source date types (datetime, date, string, NaN). Add unit tests covering each GPO's date columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Unique Key — Premier Address ID</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Premier_Key (Address ID) needs to be created in STEP and configured as the unique key for Premier entities. Until it is created, re-imports cannot match on it and will create duplicates.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Create gpo.GPO_Premier_Key attribute in STEP and mark it as the unique key before any Premier data is loaded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Unique Key — Vizient LIC</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>gpo.LIC is listed as Exists but needs to be confirmed as the unique key attribute on GPO_Top_Parent / GPO_Direct_Parent / GPO_Member object types in STEP.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Verify in STEP admin that gpo.LIC is assigned as the unique/natural key on all three GPO object types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Re-import / Idempotency</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>STEP matches on entity ID (HT_GPOID etc.) for upserts. If source IDs change between exports (e.g., GPOID reassigned), old entities will not be deleted and new duplicates will be created.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Establish a process to detect retired IDs (compare previous load list vs current) and send delete or inactivate operations to STEP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Parent Name Columns</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Top Parent Name / Direct Parent Name columns exist in source files but are not loaded as attributes — they are only used to synthesize implied parent nodes. If a parent exists in STEP with a different name, it will not be updated.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Ensure implied parent synthesis uses the name from the most authoritative row. Consider adding parent name reconciliation to the load script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Large File Performance</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>HealthTrust has 96,088 rows. Generating a single STEPXML file for all members may produce a very large file that strains STEP import. No chunking is implemented.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Add --chunk-size argument to split output into N-row STEPXML files (e.g., 10,000 rows each). Load in hierarchy order per chunk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>DEA Data — HealthTrust</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>HealthTrust source data has one row per DEA number per member. DEA numbers are stripped during deduplication and are not loaded into STEP at all.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>HealthTrust</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Confirm with business whether DEA data is required in STEP. If yes, design a member_dea child entity type and add a DEA load pass after Pass 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Attribute Data Types in STEP</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>All attributes marked Needs Creating have not had their STEP data types confirmed (Text, Date, Number, Boolean). Date fields especially must be created as Date type in STEP or values will not sort/filter correctly.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Premier, Vizient</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Before creating attributes, document required data type for each. Date fields: gpo.Affiliation_Start/End_Date_1/2/3, gpo.Membership_Eligible_Date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Error Reporting</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>The current STEPXML generator silently skips rows with missing required fields (native_member_id, top_parent_id). There is no row-level error log or summary of skipped records.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Add a skipped-rows log (CSV or printed table) that captures row index, GPOID/LIC/AddressID, and reason for skip. Helps with data quality review post-load.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Premier program date fields to Attribute Mapping sheet
Added 6 CrossReference fields that were mapped in the script but absent
from the sheet: AscenDrive, KIINDO, SURPASS Start/End Dates.
Marked blue (CrossReference) to distinguish from flat attributes —
these are emitted as STEPXML child elements requiring a STEP Reference
Type, not a simple attribute. Also added legend row at bottom of sheet.

Attribute Mapping sheet now covers all 42 fields across all three GPOs.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +72,12 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+        <bgColor rgb="00DDEEFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -81,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -97,6 +107,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2351,7 +2367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3059,482 +3075,681 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>AscenDrive Start Date</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>ascendrive_start</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>gpo.AscenDrive_Start_Date</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>AscenDrive Start Date</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>AscenDrive End Date</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>ascendrive_end</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>gpo.AscenDrive_End_Date</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>AscenDrive End Date</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>KIINDO Start Date</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>kiindo_start</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>gpo.KIINDO_Start_Date</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>KIINDO Start Date</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>KIINDO End Date</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>kiindo_end</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>gpo.KIINDO_End_Date</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>KIINDO End Date</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>SURPASS Start Date</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>surpass_start</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>gpo.SURPASS_Start_Date</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>SURPASS Start Date</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>SURPASS End Date</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>surpass_end</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>gpo.SURPASS_End_Date</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>SURPASS End Date</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>CrossReference</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 1</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>affiliation_1</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>gpo.Aggregation_Affiliation_1</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 1</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 2</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>affiliation_2</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>gpo.Aggregation_Affiliation_2</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 2</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 3</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>affiliation_3</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>gpo.Aggregation_Affiliation_3</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Aggregation Affiliation 3</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 1</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>affiliation_1_start</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_1</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 1</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 1</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>affiliation_1_end</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_1</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 1</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 2</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>affiliation_2_start</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_2</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 2</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 2</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>affiliation_2_end</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_2</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D35" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 2</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E35" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 3</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B36" s="1" t="inlineStr">
         <is>
           <t>affiliation_3_start</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C36" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_3</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D36" s="1" t="inlineStr">
         <is>
           <t>Affiliation Start Date 3</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E36" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 3</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B37" s="1" t="inlineStr">
         <is>
           <t>affiliation_3_end</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="C37" s="1" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_3</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="D37" s="1" t="inlineStr">
         <is>
           <t>Affiliation End Date 3</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="E37" s="1" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Member ID</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>vizient_member_id</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>gpo.Vizient_Member_ID</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Vizient Member ID</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>supply_program</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>gpo.Supply_Program</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>amc_tier_pricing</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>gpo.AMC_Tier_Pricing</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Needs Creating</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Vizient Group 1</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>group_1</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_1</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Vizient Group 1</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Vizient Group 2</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>group_2</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_2</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Vizient Group 2</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Exists</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Vizient Group 3</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>group_3</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>gpo.Vizient_Group_3</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Vizient Group 3</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Legend: Blue = CrossReference child record (stored as child element in STEPXML, not a flat attribute). Requires STEP Reference Type or child object type, not just an attribute.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 5 missing gaps to Potential Gaps sheet (items 16–20)
Covers questions from design review not previously captured:
- #16 Workflow/Lifecycle State (Medium)
- #17 Context/Language — context_id confirmation (High)
- #18 Delta/Refresh Strategy — monthly full replace vs incremental (High)
- #19 Inactivation — members removed from source file (High)
- #20 Mid-Load Failure/Rollback — partial state after pass failure (Medium)

Sheet now has 20 gap items total.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3960,7 +3960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4453,6 +4453,156 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Workflow / Lifecycle State</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>It is not defined whether GPO entities in STEP should have a lifecycle state (e.g. Draft, Active, Retired/Obsolete). Without this, there is no way to flag inactive or expired members in STEP separate from deleting them.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Confirm with STEP admin whether a workflow is required on GPO_Top_Parent / GPO_Direct_Parent / GPO_Member object types. If yes, define state transitions and map member_status values to STEP states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Context / Language</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>The STEPXML generator hard-codes context_id="Content". It is not confirmed whether attribute values need to be loaded in a specific STEP context or multiple contexts (e.g. for locale-specific display). If the wrong context is used, attributes may not appear in the UI.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Confirm with STEP admin the correct context ID for GPO data. If multi-context is required (e.g. EN context for display), update STEP_CONFIG["context_id"] in gpo_to_stepxml.py and re-test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Delta / Refresh Strategy</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>GPO files are typically sent monthly. It is not defined whether each load is a full replace (delete all and reload) or an incremental update (upsert changed rows only). Full replace risks data loss; incremental risks leaving stale records if IDs are retired.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Define a monthly refresh SOP: (1) compare new file IDs vs previous load IDs, (2) upsert matching IDs, (3) flag or retire IDs no longer in source. Document whether STEP receives a delete/inactivate instruction for removed members.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Inactivation — Members Removed from Source</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>If a member row disappears from a GPO source file (e.g. terminated membership), the current script has no mechanism to detect or handle this. The STEP entity will remain active with no indication it is no longer a member.</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Add a post-load comparison step: load the previous member ID list, diff against the new file, and emit an inactivate/delete STEPXML for any IDs no longer present. Alternatively set member_status to Inactive via a separate update pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Mid-Load Failure / Rollback</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Loads run across 3-4 passes (Top Parents → Direct Parents → Members → Child Records). If a pass fails halfway, the STEP database is in a partial state — some parents exist, some members do not. There is no rollback or resume mechanism in the current scripts.</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Consider wrapping each pass in a STEP workspace/sandbox so partial loads can be discarded. Alternatively, log successfully loaded entity IDs per pass so a resume-from-checkpoint can skip already-loaded rows on re-run.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Premier Address ID attribute: GPO_Premier_Key → gpo.Address_ID
Attribute already exists in STEP. Updated in:
- gpo_to_stepxml.py GPO_ATTRIBUTE_MAP (premier native_member_id)
- Attribute Mapping sheet: ID corrected, status changed to Exists
- Unique Key Design sheet: all references updated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -114,6 +114,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2206,12 +2207,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>GPO_Premier_Key</t>
+          <t>Address_ID</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>GPO_Premier_Key needs to be created in STEP</t>
+          <t>Address_ID needs to be created in STEP</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2301,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
+          <t>GPO_HealthTrust_Key / Address_ID / GPO_Vizient_Key</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2347,7 +2348,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
+          <t>GPO_HealthTrust_Key / Address_ID / GPO_Vizient_Key</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -2435,34 +2436,34 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Address ID</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>native_member_id</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>gpo.GPO_Premier_Key</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>gpo.Address_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>GPO Premier Key</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -3746,6 +3747,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Premier unique key name in Unique Key Design sheet
Key name is GPO_Premier_Key (the STEP key definition ID).
Attribute that holds the value is gpo.Address_ID (separate — updated previously).
Corrected all rows in Unique Key Design sheet that were incorrectly
showing Address_ID as the key name.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2207,12 +2207,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Address_ID</t>
+          <t>GPO_Premier_Key</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Address_ID needs to be created in STEP</t>
+          <t>Exists in STEP</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>GPO_HealthTrust_Key / Address_ID / GPO_Vizient_Key</t>
+          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>GPO_HealthTrust_Key / Address_ID / GPO_Vizient_Key</t>
+          <t>GPO_HealthTrust_Key / GPO_Premier_Key / GPO_Vizient_Key</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -3747,7 +3747,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mark gpo.Override_Name as Exists in STEP
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2564,34 +2564,34 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Override Name</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>override_name</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>gpo.Override_Name</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Override Name</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -3747,6 +3747,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add LOV Definitions sheet with LOV_Address_Type
LOV ID: LOV_Address_Type
Attribute: gpo.Address_Type (Premier)
Values: Bill To, Mail To, Ship To, Primary

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Reference Type" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Potential Gaps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="LOV Definitions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -115,6 +116,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3747,7 +3751,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>
@@ -4608,4 +4611,170 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>LOV ID</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>LOV Name</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>GPO</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>LOV_Address_Type</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>gpo.Address_Type</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Bill To</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>LOV_Address_Type</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>gpo.Address_Type</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Mail To</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>LOV_Address_Type</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>gpo.Address_Type</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Ship To</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>LOV_Address_Type</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>gpo.Address_Type</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Premier</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Attribute Mapping: gpo.Address_Type marked Exists with LOV reference
Status updated to 'Exists — LOV: LOV_Address_Type'

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2600,34 +2600,34 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Address Type</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>address_type</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>gpo.Address_Type</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Address Type</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Exists — LOV: LOV_Address_Type</t>
         </is>
       </c>
     </row>
@@ -3751,6 +3751,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mark gpo.Comments as Exists in STEP
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2920,34 +2920,34 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>comments</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>gpo.Comments</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>HealthTrust</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark gpo.Relationship_To_Top_Parent as Exists in STEP
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -2984,34 +2984,34 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Relationship to Top Parent</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>relationship_to_top_parent</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>gpo.Relationship_To_Top_Parent</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Relationship to Top Parent</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark gpo.Relationship_To_Direct_Parent as Exists in STEP
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3016,34 +3016,34 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Relationship to Direct Parent</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>relationship_to_direct_parent</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>gpo.Relationship_To_Direct_Parent</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Relationship to Direct Parent</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark 7 Premier attributes as Exists in STEP
- gpo.Affiliation_Start_Date_1/2/3
- gpo.Affiliation_End_Date_1/2/3
- gpo.Committed_Program_Eligibility

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -118,6 +118,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3048,34 +3051,34 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Committed Program Eligibility</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>committed_program_eligibility</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>gpo.Committed_Program_Eligibility</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Committed Program Eligibility</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -3368,194 +3371,194 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 1</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>affiliation_1_start</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_1</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 1</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 1</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>affiliation_1_end</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_1</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 1</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 2</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>affiliation_2_start</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_2</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 2</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 2</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>affiliation_2_end</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_2</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 2</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 3</t>
         </is>
       </c>
-      <c r="B36" s="1" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>affiliation_3_start</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_Start_Date_3</t>
         </is>
       </c>
-      <c r="D36" s="1" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>Affiliation Start Date 3</t>
         </is>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 3</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
+      <c r="B37" s="10" t="inlineStr">
         <is>
           <t>affiliation_3_end</t>
         </is>
       </c>
-      <c r="C37" s="1" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>gpo.Affiliation_End_Date_3</t>
         </is>
       </c>
-      <c r="D37" s="1" t="inlineStr">
+      <c r="D37" s="10" t="inlineStr">
         <is>
           <t>Affiliation End Date 3</t>
         </is>
       </c>
-      <c r="E37" s="1" t="inlineStr">
+      <c r="E37" s="10" t="inlineStr">
         <is>
           <t>Premier</t>
         </is>
       </c>
-      <c r="F37" s="1" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Map Vizient Member ID to gpo.GPO_Member_ID (reuse existing attribute)
No new attribute needed. vizient_member_id → gpo.GPO_Member_ID,
same attribute used by HealthTrust (GPOID) and Premier (GPO ID).
Updated ATTRIBUTE_MAP in script and Attribute Mapping sheet.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3563,34 +3563,34 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Member ID</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>vizient_member_id</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>gpo.Vizient_Member_ID</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Vizient Member ID</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>gpo.GPO_Member_ID</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>GPO Member ID</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark gpo.Supply_Program and gpo.AMC_Tier_Pricing as Exists in STEP
All attributes in Attribute Mapping sheet are now Exists — no remaining
Needs Creating items.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TaQNM4FQZUZXhciBNzMFTJ
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -3595,66 +3595,66 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>supply_program</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>gpo.Supply_Program</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>Supply Program</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>amc_tier_pricing</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>gpo.AMC_Tier_Pricing</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
         <is>
           <t>AMC Tier Pricing</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>Vizient</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Needs Creating</t>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Exists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update step_data_model.xlsx with new Vizient attributes (GLN, HIN, Facility Category, Facility Type, Rx Group)
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hierarchy Structure" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Object Types" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Attributes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Load Order" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Reference Type" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Potential Gaps" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="LOV Definitions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hierarchy Structure" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object Types" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attributes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Load Order" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unique Key Design" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attribute Mapping" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Type" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Potential Gaps" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LOV Definitions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1087,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1782,6 +1782,166 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>Stores LIC — gpo.LIC — exists in STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>gpo.GLN</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GLN</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>gpo.HIN</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HIN</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Exists in STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>gpo.Facility_Category</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Facility Category</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Created in STEP</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>gpo.Facility_Type</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Facility Type</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Pending confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gpo.Rx_Group</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Rx Group</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Created in STEP</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3725,22 +3885,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vizient Group 3</t>
+          <t>GLN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>group_3</t>
+          <t>gln</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>gpo.Vizient_Group_3</t>
+          <t>gpo.GLN</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Vizient Group 3</t>
+          <t>GLN</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3754,9 +3914,136 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>HIN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>hin</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>gpo.HIN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>HIN</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Exists</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Facility Category</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>facility_category</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>gpo.Facility_Category</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Facility Category</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Facility Type</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>facility_type</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>gpo.Facility_Type</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Facility Type</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Rx Group</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>rx_group</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>gpo.Rx_Group</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Rx Group</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Vizient</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Legend: Blue = CrossReference child record (stored as child element in STEPXML, not a flat attribute). Requires STEP Reference Type or child object type, not just an attribute.</t>
         </is>

</xml_diff>

<commit_message>
Mark gpo.Facility_Type as Exists in STEP
</commit_message>
<xml_diff>
--- a/step_data_model.xlsx
+++ b/step_data_model.xlsx
@@ -1909,7 +1909,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Pending confirmation</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Exists</t>
         </is>
       </c>
     </row>
@@ -4042,6 +4042,7 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>

</xml_diff>